<commit_message>
Polish UI/copy and fix skill % rounding
- Skill progress %: use floor instead of round to match in-game display
- Home: redesign cards (no descriptions, gradient text shadow on titles)
  and tighten intro to one short sentence
- BoxChecker: drop search/filter, keep reset button only;
  shorten cost panel labels (残りガチャ回数 / 1回の◯◯ / ◯◯稼ぎ効率を計算)
- Efficiency: shorten +Coin and medal cap notices, drop 達成日数 verbosity,
  switch アイテム grid to 3x2, fix stopwatch overflow on mobile,
  rename 1日あたりの収入 → 1日あたりの稼ぎ
- Mobile readability: nowrap key Japanese phrases to avoid mid-word breaks
- Notice texts (3 BOX pages): shorten to ※「ならびかえ」→「リリース順」がおすすめ。
- Data: rename サリー → サリー(モンスターズ・インク),
  mark ダグ and ラーヤ＋ as 今月のツム,
  swap ルカ・パグーロ/メイリン・リー display order
- Regenerate ガチャデータ.xlsx to reflect data changes

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ガチャデータ.xlsx
+++ b/data/ガチャデータ.xlsx
@@ -1674,59 +1674,59 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
+      <c r="A22" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>pp-021</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>ダグ</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="E22" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G22" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="H22" s="2" t="n">
+      <c r="E22" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H22" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="I22" s="2" t="n">
+      <c r="I22" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="J22" s="2">
+      <c r="J22" s="5">
         <f>IF(COUNT(E22:I22)=5,SUM(E22:I22),"")</f>
         <v/>
       </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>VERIFIED</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="L22" s="7" t="inlineStr">
         <is>
           <t>https://game8.jp/tsumtsum/786555</t>
         </is>
       </c>
-      <c r="M22" s="4" t="inlineStr">
+      <c r="M22" s="7" t="inlineStr">
         <is>
           <t>https://xn--bdka7fb.jp/202431.html</t>
         </is>
       </c>
-      <c r="N22" s="3" t="inlineStr"/>
+      <c r="N22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
@@ -1847,59 +1847,59 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
+      <c r="A25" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>pp-024</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>ラーヤ＋</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="E25" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G25" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="H25" s="2" t="n">
+      <c r="E25" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H25" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="I25" s="2" t="n">
+      <c r="I25" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="J25" s="2">
+      <c r="J25" s="5">
         <f>IF(COUNT(E25:I25)=5,SUM(E25:I25),"")</f>
         <v/>
       </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>VERIFIED</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="L25" s="7" t="inlineStr">
         <is>
           <t>https://game8.jp/tsumtsum/789307</t>
         </is>
       </c>
-      <c r="M25" s="4" t="inlineStr">
+      <c r="M25" s="7" t="inlineStr">
         <is>
           <t>https://xn--bdka7fb.jp/202925.html</t>
         </is>
       </c>
-      <c r="N25" s="3" t="inlineStr"/>
+      <c r="N25" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:N25"/>
@@ -7879,12 +7879,12 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>p-133</t>
+          <t>p-132</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
-          <t>メイリン・リー</t>
+          <t>ルカ・パグーロ</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -7918,7 +7918,7 @@
       </c>
       <c r="L121" s="4" t="inlineStr">
         <is>
-          <t>https://xn--bdka7fb.jp/142187.html</t>
+          <t>https://xn--bdka7fb.jp/142185.html</t>
         </is>
       </c>
     </row>
@@ -7928,12 +7928,12 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>p-132</t>
+          <t>p-133</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
         <is>
-          <t>ルカ・パグーロ</t>
+          <t>メイリン・リー</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
@@ -7967,7 +7967,7 @@
       </c>
       <c r="L122" s="4" t="inlineStr">
         <is>
-          <t>https://xn--bdka7fb.jp/142185.html</t>
+          <t>https://xn--bdka7fb.jp/142187.html</t>
         </is>
       </c>
     </row>

</xml_diff>